<commit_message>
Finish Table & Form excercise
</commit_message>
<xml_diff>
--- a/HN-C0626L1-Jv111+Jv113 [BC Java Backend] TKB Module 1_Programming Foundations.xlsx
+++ b/HN-C0626L1-Jv111+Jv113 [BC Java Backend] TKB Module 1_Programming Foundations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code Gym\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B3EBAC-8431-4382-B612-5B46EE23556F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51676C9-AA25-4773-A38F-15B519625EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="393">
   <si>
     <t>THỜI KHOÁ BIỂU MODULE</t>
   </si>
@@ -1285,6 +1285,9 @@
   <si>
     <t>Không có báo cáo nào cả</t>
   </si>
+  <si>
+    <t>Học form vs table</t>
+  </si>
 </sst>
 </file>
 
@@ -1998,10 +2001,6 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2014,6 +2013,10 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2717,7 +2720,7 @@
       <c r="F13" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G13" s="110"/>
+      <c r="G13" s="108"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -2752,7 +2755,7 @@
       <c r="F14" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G14" s="110"/>
+      <c r="G14" s="108"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -2787,7 +2790,7 @@
       <c r="F15" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G15" s="110"/>
+      <c r="G15" s="108"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -2824,7 +2827,7 @@
       <c r="F16" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G16" s="113" t="s">
+      <c r="G16" s="111" t="s">
         <v>391</v>
       </c>
       <c r="H16" s="1"/>
@@ -2861,10 +2864,10 @@
       <c r="F17" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G17" s="113" t="s">
+      <c r="G17" s="111" t="s">
         <v>390</v>
       </c>
-      <c r="H17" s="112"/>
+      <c r="H17" s="110"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -2898,7 +2901,9 @@
       <c r="F18" s="105" t="s">
         <v>386</v>
       </c>
-      <c r="G18" s="110"/>
+      <c r="G18" s="111" t="s">
+        <v>392</v>
+      </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -2933,7 +2938,7 @@
         <v>31</v>
       </c>
       <c r="F19" s="103"/>
-      <c r="G19" s="110"/>
+      <c r="G19" s="108"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -2966,7 +2971,7 @@
       </c>
       <c r="E20" s="101"/>
       <c r="F20" s="103"/>
-      <c r="G20" s="110"/>
+      <c r="G20" s="108"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -2999,7 +3004,7 @@
       </c>
       <c r="E21" s="101"/>
       <c r="F21" s="103"/>
-      <c r="G21" s="110"/>
+      <c r="G21" s="108"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -3034,7 +3039,7 @@
         <v>31</v>
       </c>
       <c r="F22" s="103"/>
-      <c r="G22" s="110"/>
+      <c r="G22" s="108"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -3067,7 +3072,7 @@
       </c>
       <c r="E23" s="101"/>
       <c r="F23" s="103"/>
-      <c r="G23" s="110"/>
+      <c r="G23" s="108"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -3102,7 +3107,7 @@
         <v>47</v>
       </c>
       <c r="F24" s="104"/>
-      <c r="G24" s="110"/>
+      <c r="G24" s="108"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -3137,7 +3142,7 @@
         <v>31</v>
       </c>
       <c r="F25" s="104"/>
-      <c r="G25" s="110"/>
+      <c r="G25" s="108"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
@@ -3170,7 +3175,7 @@
       </c>
       <c r="E26" s="101"/>
       <c r="F26" s="103"/>
-      <c r="G26" s="110"/>
+      <c r="G26" s="108"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
@@ -3203,7 +3208,7 @@
       </c>
       <c r="E27" s="101"/>
       <c r="F27" s="103"/>
-      <c r="G27" s="110"/>
+      <c r="G27" s="108"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
@@ -3238,7 +3243,7 @@
         <v>31</v>
       </c>
       <c r="F28" s="103"/>
-      <c r="G28" s="110"/>
+      <c r="G28" s="108"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
@@ -3271,7 +3276,7 @@
       </c>
       <c r="E29" s="101"/>
       <c r="F29" s="103"/>
-      <c r="G29" s="110"/>
+      <c r="G29" s="108"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
@@ -3304,7 +3309,7 @@
       </c>
       <c r="E30" s="101"/>
       <c r="F30" s="103"/>
-      <c r="G30" s="110"/>
+      <c r="G30" s="108"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
@@ -3339,7 +3344,7 @@
         <v>31</v>
       </c>
       <c r="F31" s="103"/>
-      <c r="G31" s="110"/>
+      <c r="G31" s="108"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
@@ -3372,7 +3377,7 @@
       </c>
       <c r="E32" s="101"/>
       <c r="F32" s="103"/>
-      <c r="G32" s="110"/>
+      <c r="G32" s="108"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
@@ -3405,7 +3410,7 @@
       </c>
       <c r="E33" s="101"/>
       <c r="F33" s="103"/>
-      <c r="G33" s="110"/>
+      <c r="G33" s="108"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
@@ -3438,7 +3443,7 @@
       </c>
       <c r="E34" s="101"/>
       <c r="F34" s="103"/>
-      <c r="G34" s="111"/>
+      <c r="G34" s="109"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
@@ -3473,7 +3478,7 @@
         <v>70</v>
       </c>
       <c r="F35" s="103"/>
-      <c r="G35" s="111"/>
+      <c r="G35" s="109"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
@@ -3508,7 +3513,7 @@
         <v>72</v>
       </c>
       <c r="F36" s="103"/>
-      <c r="G36" s="111"/>
+      <c r="G36" s="109"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
@@ -3543,7 +3548,7 @@
         <v>74</v>
       </c>
       <c r="F37" s="103"/>
-      <c r="G37" s="110"/>
+      <c r="G37" s="108"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
@@ -3578,7 +3583,7 @@
         <v>77</v>
       </c>
       <c r="F38" s="103"/>
-      <c r="G38" s="110"/>
+      <c r="G38" s="108"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
@@ -3613,7 +3618,7 @@
         <v>80</v>
       </c>
       <c r="F39" s="103"/>
-      <c r="G39" s="110"/>
+      <c r="G39" s="108"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
@@ -25871,10 +25876,10 @@
       <c r="A7" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="B7" s="108" t="s">
+      <c r="B7" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="109"/>
+      <c r="C7" s="113"/>
       <c r="D7" s="32" t="s">
         <v>91</v>
       </c>
@@ -25900,10 +25905,10 @@
       <c r="A8" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="108" t="s">
+      <c r="B8" s="112" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="109"/>
+      <c r="C8" s="113"/>
       <c r="D8" s="32" t="s">
         <v>97</v>
       </c>
@@ -25929,10 +25934,10 @@
       <c r="A9" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="108" t="s">
+      <c r="B9" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="C9" s="109"/>
+      <c r="C9" s="113"/>
       <c r="D9" s="38"/>
       <c r="E9" s="33" t="s">
         <v>103</v>
@@ -25956,10 +25961,10 @@
       <c r="A10" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="B10" s="108" t="s">
+      <c r="B10" s="112" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="109"/>
+      <c r="C10" s="113"/>
       <c r="D10" s="32" t="s">
         <v>108</v>
       </c>
@@ -34287,10 +34292,10 @@
       <c r="A6" s="32" t="s">
         <v>373</v>
       </c>
-      <c r="B6" s="108" t="s">
+      <c r="B6" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="109"/>
+      <c r="C6" s="113"/>
       <c r="D6" s="32" t="s">
         <v>91</v>
       </c>
@@ -34314,10 +34319,10 @@
       <c r="A7" s="32" t="s">
         <v>376</v>
       </c>
-      <c r="B7" s="108" t="s">
+      <c r="B7" s="112" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="109"/>
+      <c r="C7" s="113"/>
       <c r="D7" s="32" t="s">
         <v>97</v>
       </c>
@@ -34340,10 +34345,10 @@
       <c r="A8" s="32" t="s">
         <v>380</v>
       </c>
-      <c r="B8" s="108" t="s">
+      <c r="B8" s="112" t="s">
         <v>381</v>
       </c>
-      <c r="C8" s="109"/>
+      <c r="C8" s="113"/>
       <c r="D8" s="32" t="s">
         <v>108</v>
       </c>

</xml_diff>